<commit_message>
feat: handle panipat/panchkula data update and enable password change
</commit_message>
<xml_diff>
--- a/TESTING COURT EXCEL FILE/court portal data PANIPAT.xlsx
+++ b/TESTING COURT EXCEL FILE/court portal data PANIPAT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\court portal antigravity\TESTING COURT EXCEL FILE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FC67954-61DB-48E1-8923-EFA25D8DCF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B773169-0772-4B32-93BF-4C4B7221B3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="19386" windowHeight="11466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="82">
   <si>
     <t>district</t>
   </si>
@@ -211,9 +211,6 @@
     <t>Balraj</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Ms Anandita Bhargava</t>
   </si>
   <si>
@@ -266,21 +263,6 @@
   </si>
   <si>
     <t>Ms Varsha Sharma</t>
-  </si>
-  <si>
-    <t>Utility Court</t>
-  </si>
-  <si>
-    <t>Consumer Commission /Labour Office Court/ SDM/CTM/Executive Court/Any Authority</t>
-  </si>
-  <si>
-    <t>Joginder Pal</t>
-  </si>
-  <si>
-    <t>Commissioner /DM</t>
-  </si>
-  <si>
-    <t>HC/EASI</t>
   </si>
   <si>
     <t>LD. CJM cum Secretary (DLSA) SMK</t>
@@ -561,7 +543,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H1000"/>
+  <dimension ref="A1:H997"/>
   <sheetFormatPr defaultColWidth="12.64453125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="6.703125" bestFit="1" customWidth="1"/>
@@ -615,10 +597,10 @@
         <v>10</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H2" s="4">
         <v>9416530661</v>
@@ -639,10 +621,10 @@
         <v>14</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H3" s="4">
         <v>9053300939</v>
@@ -663,10 +645,10 @@
         <v>14</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="H4" s="4">
         <v>9416567587</v>
@@ -687,10 +669,10 @@
         <v>14</v>
       </c>
       <c r="F5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H5" s="4">
         <v>9813602612</v>
@@ -711,10 +693,10 @@
         <v>22</v>
       </c>
       <c r="F6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H6" s="4">
         <v>9055232341</v>
@@ -735,10 +717,10 @@
         <v>25</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H7" s="4">
         <v>7988887228</v>
@@ -759,10 +741,10 @@
         <v>14</v>
       </c>
       <c r="F8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H8" s="4">
         <v>8950377711</v>
@@ -783,10 +765,10 @@
         <v>30</v>
       </c>
       <c r="F9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="H9" s="4">
         <v>9080400937</v>
@@ -807,10 +789,10 @@
         <v>30</v>
       </c>
       <c r="F10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="H10" s="4">
         <v>7830529831</v>
@@ -831,10 +813,10 @@
         <v>37</v>
       </c>
       <c r="F11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="H11" s="4">
         <v>9050449499</v>
@@ -855,10 +837,10 @@
         <v>40</v>
       </c>
       <c r="F12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H12" s="4">
         <v>9812913130</v>
@@ -879,10 +861,10 @@
         <v>43</v>
       </c>
       <c r="F13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H13" s="4">
         <v>9896693927</v>
@@ -903,10 +885,10 @@
         <v>46</v>
       </c>
       <c r="F14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H14" s="4">
         <v>9729640500</v>
@@ -927,10 +909,10 @@
         <v>49</v>
       </c>
       <c r="F15" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="H15" s="4">
         <v>9050703033</v>
@@ -951,10 +933,10 @@
         <v>53</v>
       </c>
       <c r="F16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="H16" s="4">
         <v>9992935855</v>
@@ -975,10 +957,10 @@
         <v>49</v>
       </c>
       <c r="F17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="H17" s="4">
         <v>9034834348</v>
@@ -999,10 +981,10 @@
         <v>53</v>
       </c>
       <c r="F18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="H18" s="4">
         <v>9896381052</v>
@@ -1023,10 +1005,10 @@
         <v>53</v>
       </c>
       <c r="F19" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="H19" s="4">
         <v>9050419747</v>
@@ -1047,10 +1029,10 @@
         <v>53</v>
       </c>
       <c r="F20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="H20" s="4">
         <v>9991107616</v>
@@ -1060,21 +1042,19 @@
       <c r="A21" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>53</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="H21" s="4">
         <v>9812596121</v>
@@ -1084,21 +1064,19 @@
       <c r="A22" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>53</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="H22" s="4">
         <v>7837337473</v>
@@ -1108,21 +1086,19 @@
       <c r="A23" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>53</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="H23" s="4">
         <v>8168138955</v>
@@ -1137,16 +1113,16 @@
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>72</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H24" s="4">
         <v>9896071111</v>
@@ -1161,16 +1137,16 @@
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="H25" s="4">
         <v>9518163196</v>
@@ -1185,16 +1161,16 @@
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="H26" s="4">
         <v>9050400760</v>
@@ -1204,21 +1180,19 @@
       <c r="A27" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G27" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="H27" s="4">
         <v>8095244353</v>
@@ -1228,89 +1202,25 @@
       <c r="A28" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E28" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>63</v>
-      </c>
       <c r="G28" s="3"/>
-      <c r="H28" s="4" t="s">
-        <v>63</v>
-      </c>
+      <c r="H28" s="4"/>
     </row>
     <row r="29" spans="1:8" ht="12.7" x14ac:dyDescent="0.4">
-      <c r="A29" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="G29" s="3"/>
-      <c r="H29" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="50.7" x14ac:dyDescent="0.4">
-      <c r="A30" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="H30" s="4">
-        <v>9991070455</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="25.35" x14ac:dyDescent="0.4">
-      <c r="A31" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="H31" s="4">
-        <v>9991070455</v>
-      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:8" ht="12.7" x14ac:dyDescent="0.4">
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:8" ht="12.7" x14ac:dyDescent="0.4">
+      <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:8" ht="12.7" x14ac:dyDescent="0.4">
       <c r="F32" s="1"/>
@@ -4210,18 +4120,9 @@
     <row r="997" spans="6:6" ht="12.7" x14ac:dyDescent="0.4">
       <c r="F997" s="1"/>
     </row>
-    <row r="998" spans="6:6" ht="12.7" x14ac:dyDescent="0.4">
-      <c r="F998" s="1"/>
-    </row>
-    <row r="999" spans="6:6" ht="12.7" x14ac:dyDescent="0.4">
-      <c r="F999" s="1"/>
-    </row>
-    <row r="1000" spans="6:6" ht="12.7" x14ac:dyDescent="0.4">
-      <c r="F1000" s="1"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F1 F32:F1000" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F1 F29:F997" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"naib court rank,Insp,PSI,SI,ASI/ESI,ASI,HC/ESI,HC/EASI,HC,C-1/EHC,C-1,C-1/ORPSI,CT/ESI,CT/EASI,CT/EHC/ORPHC,CT/EHC,CT,R/CT,SPO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>